<commit_message>
feat: implementar estilo visual OriginLab Pro com ticks internos, caixa fechada e paleta cientifica
</commit_message>
<xml_diff>
--- a/dados_e_graficos_bosque.xlsx
+++ b/dados_e_graficos_bosque.xlsx
@@ -318,7 +318,7 @@
         <axId val="100"/>
         <scaling>
           <orientation val="minMax"/>
-          <max val="32"/>
+          <max val="33"/>
           <min val="24"/>
         </scaling>
         <axPos val="l"/>
@@ -504,7 +504,7 @@
         <axId val="100"/>
         <scaling>
           <orientation val="minMax"/>
-          <max val="32"/>
+          <max val="33"/>
           <min val="24"/>
         </scaling>
         <axPos val="l"/>
@@ -690,7 +690,7 @@
         <axId val="100"/>
         <scaling>
           <orientation val="minMax"/>
-          <max val="32"/>
+          <max val="33"/>
           <min val="22"/>
         </scaling>
         <axPos val="l"/>

</xml_diff>